<commit_message>
Fix inserts input and fatigue
</commit_message>
<xml_diff>
--- a/tests/bolts/res/M12_insert.xlsx
+++ b/tests/bolts/res/M12_insert.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cassy\tests\bolts\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5153AD3-6E46-45F7-923B-E8CC65FA14D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A6E7D8-9FDD-4590-A9A9-B02E88CC0FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1380" windowWidth="29040" windowHeight="15840" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
   </bookViews>
   <sheets>
     <sheet name="Insert Data" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>Dimensions of the bolts and assembled parts</t>
   </si>
@@ -97,24 +97,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>1</t>
-    </r>
-  </si>
-  <si>
-    <t>diameter of smooth shank</t>
-  </si>
-  <si>
-    <r>
-      <t>d</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="subscript"/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t>f</t>
     </r>
   </si>
@@ -126,24 +108,6 @@
   </si>
   <si>
     <t>minor diameter of tapping</t>
-  </si>
-  <si>
-    <r>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="subscript"/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>p</t>
-    </r>
-  </si>
-  <si>
-    <t>diameter of drilling circle</t>
   </si>
   <si>
     <r>
@@ -167,24 +131,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>mean diameter under head</t>
-  </si>
-  <si>
-    <r>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="subscript"/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>m</t>
-    </r>
-  </si>
-  <si>
     <t>Material name</t>
   </si>
   <si>
@@ -198,12 +144,6 @@
   </si>
   <si>
     <t>friction coefficient between engaged threads</t>
-  </si>
-  <si>
-    <t>f_prime</t>
-  </si>
-  <si>
-    <t>friction coefficient under head</t>
   </si>
   <si>
     <t>d_vh</t>
@@ -289,7 +229,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -543,19 +483,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="dotted">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -601,7 +528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -660,15 +587,24 @@
     <xf numFmtId="2" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -676,18 +612,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -720,7 +644,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>74351</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>50233</xdr:rowOff>
+      <xdr:rowOff>116908</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -757,13 +681,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>107008</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>34685</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>57375</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>121541</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -801,13 +725,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>635999</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>152944</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>473886</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -845,13 +769,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>249282</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>59</xdr:row>
       <xdr:rowOff>78540</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1185,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C53422B0-ED6B-49AF-B1B2-2F7C5139E7C1}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" style="2" customWidth="1"/>
@@ -1196,12 +1120,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="28"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -1302,7 +1226,6 @@
         <v>13</v>
       </c>
       <c r="C6" s="18">
-        <f>C4</f>
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -1316,15 +1239,15 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="18">
-        <v>12</v>
+      <c r="C7" s="19">
+        <v>11.43</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -1337,7 +1260,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1345,7 +1268,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="19">
-        <v>11.43</v>
+        <v>60</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -1358,18 +1281,17 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="19">
-        <f>C4+1</f>
-        <v>13</v>
-      </c>
-      <c r="D9" s="5" t="s">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="24">
+        <v>0</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="1"/>
@@ -1380,18 +1302,18 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="18">
-        <v>13.7</v>
+      <c r="C10" s="21">
+        <v>0.15</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1401,18 +1323,18 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="19">
-        <v>60</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>7</v>
+      <c r="D11" s="16" t="s">
+        <v>18</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1423,18 +1345,10 @@
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="28">
-        <v>0</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>7</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -1444,18 +1358,10 @@
       <c r="K12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="22">
-        <v>0.15</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>22</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -1464,17 +1370,11 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="15">
-        <v>0.15</v>
-      </c>
-      <c r="D14" s="20"/>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -1483,19 +1383,11 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>22</v>
-      </c>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -1517,58 +1409,6 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -1579,6 +1419,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100EFE0C39B20CFE747B2EDBEF1A424A9C1" ma:contentTypeVersion="14" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="fc5d43efe255f0326fdf88779d9e8cc0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71e126cb-1963-4e7b-b13a-15d2f64f78e9" xmlns:ns3="f41f4605-e15c-4135-bd96-d3970596b173" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c67b044c92a952204dd5da40bf3ff3c1" ns2:_="" ns3:_="">
     <xsd:import namespace="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
@@ -1807,15 +1656,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1828,6 +1668,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AD0DBB6-51A1-41E4-B899-7133D1D7DFCB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1846,14 +1694,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B53875E3-DFDB-4F02-8AAC-AEAA1E089733}">
   <ds:schemaRefs>

</xml_diff>